<commit_message>
ng: update lab forms
</commit_message>
<xml_diff>
--- a/ONCHO/Entomological survey Survey/Nigeria/2026/ng_oncho_2601_4_b_lab_tar.xlsx
+++ b/ONCHO/Entomological survey Survey/Nigeria/2026/ng_oncho_2601_4_b_lab_tar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\ONCHO\Entomological survey Survey\Nigeria\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{779D2E7C-D549-4C10-84D3-4E1157334EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55E796E-F70C-4EBC-946C-97115F6608EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -322,9 +322,6 @@
     <t>PCR ELISA</t>
   </si>
   <si>
-    <t>select_multiple type_test</t>
-  </si>
-  <si>
     <t>BAC</t>
   </si>
   <si>
@@ -442,10 +439,13 @@
     <t>13. Number of heads in Pool #${pool_idx}</t>
   </si>
   <si>
-    <t>. &lt;= 200</t>
-  </si>
-  <si>
-    <t>The number of pools is limited to 200</t>
+    <t>select_one type_test</t>
+  </si>
+  <si>
+    <t>. &gt; 0 and . &lt;= 200</t>
+  </si>
+  <si>
+    <t>The number of pools must between 1 and 200 inclusive</t>
   </si>
 </sst>
 </file>
@@ -1283,10 +1283,10 @@
         <v>20</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
@@ -1316,13 +1316,13 @@
     </row>
     <row r="4" spans="1:26" s="18" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -1352,13 +1352,13 @@
     </row>
     <row r="5" spans="1:26" s="18" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="22" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -1394,7 +1394,7 @@
         <v>34</v>
       </c>
       <c r="C6" s="28" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D6" s="28"/>
       <c r="E6" s="26"/>
@@ -1418,7 +1418,7 @@
         <v>56</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D7" s="28"/>
       <c r="E7" s="26"/>
@@ -1441,10 +1441,10 @@
         <v>65</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C8" s="28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D8" s="28"/>
       <c r="E8" s="26"/>
@@ -1464,13 +1464,13 @@
     </row>
     <row r="9" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B9" s="27" t="s">
         <v>57</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D9" s="28"/>
       <c r="E9" s="26"/>
@@ -1494,7 +1494,7 @@
         <v>36</v>
       </c>
       <c r="C10" s="28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D10" s="28"/>
       <c r="E10" s="26"/>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="K10" s="26"/>
       <c r="L10" s="26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M10" s="26"/>
       <c r="N10" s="26"/>
@@ -1520,7 +1520,7 @@
         <v>58</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D11" s="28" t="s">
         <v>59</v>
@@ -1543,19 +1543,15 @@
         <v>20</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C12" s="28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D12" s="28"/>
       <c r="E12" s="26"/>
-      <c r="F12" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="G12" s="28" t="s">
-        <v>136</v>
-      </c>
+      <c r="F12" s="26"/>
+      <c r="G12" s="28"/>
       <c r="H12" s="26"/>
       <c r="I12" s="26"/>
       <c r="J12" s="26" t="s">
@@ -1587,15 +1583,15 @@
       <c r="L13" s="29"/>
       <c r="M13" s="29"/>
       <c r="N13" s="29" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B14" s="27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C14" s="28"/>
       <c r="D14" s="28"/>
@@ -1604,7 +1600,7 @@
       <c r="G14" s="28"/>
       <c r="H14" s="26"/>
       <c r="I14" s="26" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J14" s="26"/>
       <c r="K14" s="26"/>
@@ -1612,15 +1608,15 @@
       <c r="M14" s="26"/>
       <c r="N14" s="26"/>
     </row>
-    <row r="15" spans="1:26" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
       <c r="B15" s="27" t="s">
         <v>93</v>
       </c>
       <c r="C15" s="28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D15" s="28"/>
       <c r="E15" s="26"/>
@@ -1636,20 +1632,24 @@
       <c r="M15" s="26"/>
       <c r="N15" s="26"/>
     </row>
-    <row r="16" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C16" s="28" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D16" s="28"/>
       <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="28"/>
+      <c r="F16" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>136</v>
+      </c>
       <c r="H16" s="26"/>
       <c r="I16" s="26"/>
       <c r="J16" s="26" t="s">
@@ -1662,20 +1662,20 @@
     </row>
     <row r="17" spans="1:14" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D17" s="28"/>
       <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="28"/>
       <c r="H17" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I17" s="26"/>
       <c r="J17" s="26" t="s">
@@ -1688,13 +1688,13 @@
     </row>
     <row r="18" spans="1:14" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B18" s="27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C18" s="28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D18" s="28"/>
       <c r="E18" s="26"/>
@@ -1712,20 +1712,20 @@
     </row>
     <row r="19" spans="1:14" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C19" s="28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D19" s="28"/>
       <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="28"/>
       <c r="H19" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I19" s="26"/>
       <c r="J19" s="26"/>
@@ -1742,7 +1742,7 @@
         <v>24</v>
       </c>
       <c r="C20" s="28" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D20" s="28"/>
       <c r="E20" s="26"/>
@@ -1751,7 +1751,7 @@
       <c r="H20" s="26"/>
       <c r="I20" s="26"/>
       <c r="J20" s="26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K20" s="26"/>
       <c r="L20" s="26"/>
@@ -1989,10 +1989,10 @@
         <v>76</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E13" t="s">
         <v>61</v>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="D24" s="13"/>
       <c r="F24" s="21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -2366,7 +2366,7 @@
         <v>33</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>94</v>
@@ -2393,19 +2393,19 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B46" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="B46" s="20" t="s">
-        <v>99</v>
-      </c>
       <c r="C46" s="20" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D46" s="13"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>27</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B48" s="12" t="s">
         <v>28</v>
@@ -2429,7 +2429,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B49" s="12" t="s">
         <v>26</v>

</xml_diff>